<commit_message>
Dataset checkpoint: 34 benchmark items (was 22); +12 promoted from all-platform sourcing this session
</commit_message>
<xml_diff>
--- a/research/dataset/TruthLens_Dataset.xlsx
+++ b/research/dataset/TruthLens_Dataset.xlsx
@@ -469,7 +469,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-07T15:17:01+00:00</t>
+          <t>2026-09-07T15:38:20+00:00</t>
         </is>
       </c>
     </row>
@@ -481,7 +481,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>a4b03af</t>
+          <t>9ab9768</t>
         </is>
       </c>
     </row>
@@ -688,14 +688,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK27"/>
+  <dimension ref="A1:AK35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="23" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
     <col width="60" customWidth="1" min="8" max="8"/>
@@ -3673,6 +3673,870 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>item-0027</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>validation</t>
+        </is>
+      </c>
+      <c r="D28" t="b">
+        <v>1</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>cand-ap-altnews-0196</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>facebook</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/reel/4194321227564873</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>https://www.altnews.in/west-asia-conflict-old-video-falsely-viral-as-footage-from-tel-aviv-after-iranian-strike/</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>Israel occupied schools and hospitals, killing 160 Iranian school girls</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>altnews.in</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>https://www.altnews.in/west-asia-conflict-old-video-falsely-viral-as-footage-from-tel-aviv-after-iranian-strike/</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>provenance</t>
+        </is>
+      </c>
+      <c r="V28" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="W28" t="b">
+        <v>1</v>
+      </c>
+      <c r="X28" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y28" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z28" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD28" t="b">
+        <v>1</v>
+      </c>
+      <c r="AF28" t="inlineStr">
+        <is>
+          <t>3a03a21e6b7074a92d5b7fb12a2a833e76c4f2a5f65cf4d272428b2310b98250</t>
+        </is>
+      </c>
+      <c r="AJ28" t="inlineStr">
+        <is>
+          <t>candidates_v3_altnews.jsonl</t>
+        </is>
+      </c>
+      <c r="AK28" t="inlineStr">
+        <is>
+          <t>2026-09-07T13:51:43.696587+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>item-0028</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>validation</t>
+        </is>
+      </c>
+      <c r="D29" t="b">
+        <v>1</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>cand-ap-altnews-0316</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>https://twitter.com/pathan_sumaya/status/2015708362789556721</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>https://www.altnews.in/video-from-bangladesh-of-man-popping-childs-balloons-falsely-shared-with-communal-angle/</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>A person who is doing brutality against a Muslim balloon seller or a crowd instead of helping takes a video?</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>altnews.in</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>https://www.altnews.in/video-from-bangladesh-of-man-popping-childs-balloons-falsely-shared-with-communal-angle/</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>provenance</t>
+        </is>
+      </c>
+      <c r="V29" t="n">
+        <v>0.9999</v>
+      </c>
+      <c r="W29" t="b">
+        <v>1</v>
+      </c>
+      <c r="X29" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y29" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z29" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD29" t="b">
+        <v>1</v>
+      </c>
+      <c r="AF29" t="inlineStr">
+        <is>
+          <t>ce0e74bf0e7f76bf93acfd65bd4ba62b751ff8a7e151d304ca05a7bc178c4da3</t>
+        </is>
+      </c>
+      <c r="AJ29" t="inlineStr">
+        <is>
+          <t>candidates_v3_altnews.jsonl</t>
+        </is>
+      </c>
+      <c r="AK29" t="inlineStr">
+        <is>
+          <t>2026-09-07T14:08:54.320547+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>item-0029</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>validation</t>
+        </is>
+      </c>
+      <c r="D30" t="b">
+        <v>1</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>cand-ap-altnews-0382</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>https://twitter.com/yoursurajnaik/status/1997721155235713176</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>https://www.altnews.in/old-video-of-aviation-minister-k-r-naidu-dancing-falsely-viral-amid-indigo-crisis/</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>This government has mastered one thing: entertainment over governance.</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>altnews.in</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>https://www.altnews.in/old-video-of-aviation-minister-k-r-naidu-dancing-falsely-viral-amid-indigo-crisis/</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>provenance</t>
+        </is>
+      </c>
+      <c r="V30" t="n">
+        <v>1</v>
+      </c>
+      <c r="W30" t="b">
+        <v>1</v>
+      </c>
+      <c r="X30" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y30" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z30" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD30" t="b">
+        <v>1</v>
+      </c>
+      <c r="AF30" t="inlineStr">
+        <is>
+          <t>127ecea126d89ac271dab414e69d52e400ae5876abe319897479152099993014</t>
+        </is>
+      </c>
+      <c r="AJ30" t="inlineStr">
+        <is>
+          <t>candidates_v3_altnews.jsonl</t>
+        </is>
+      </c>
+      <c r="AK30" t="inlineStr">
+        <is>
+          <t>2026-09-07T14:15:35.466818+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>item-0030</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>validation</t>
+        </is>
+      </c>
+      <c r="D31" t="b">
+        <v>1</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>cand-ap-altnews-0407</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>https://twitter.com/rvaidya2000/status/1995691015437713467</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>https://www.altnews.in/video-of-udhayanidhi-stalin-using-computer-without-switching-it-on-is-ai-generated/</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>He's so brilliant that he can work on a computer even without switching it on!</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>altnews.in</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>https://www.altnews.in/video-of-udhayanidhi-stalin-using-computer-without-switching-it-on-is-ai-generated/</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>provenance</t>
+        </is>
+      </c>
+      <c r="V31" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="W31" t="b">
+        <v>1</v>
+      </c>
+      <c r="X31" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y31" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z31" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD31" t="b">
+        <v>1</v>
+      </c>
+      <c r="AF31" t="inlineStr">
+        <is>
+          <t>37b3dc508f0e042df4bb597d4596bfb17c69cac6a7a290fe533a456b175974d9</t>
+        </is>
+      </c>
+      <c r="AJ31" t="inlineStr">
+        <is>
+          <t>candidates_v3_altnews.jsonl</t>
+        </is>
+      </c>
+      <c r="AK31" t="inlineStr">
+        <is>
+          <t>2026-09-07T14:19:08.313987+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>item-0031</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>validation</t>
+        </is>
+      </c>
+      <c r="D32" t="b">
+        <v>1</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>cand-ap-altnews-0522</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>https://twitter.com/MrSinha_/status/1983456538309317021</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>https://www.altnews.in/no-rahul-gandhi-did-not-call-chhath-puja-a-drama-claim-by-modi-bjp-camp-false/</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>Rahul Gandhi called Chhath Puja 'drama'</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>altnews.in</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>https://www.altnews.in/no-rahul-gandhi-did-not-call-chhath-puja-a-drama-claim-by-modi-bjp-camp-false/</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>provenance</t>
+        </is>
+      </c>
+      <c r="V32" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="W32" t="b">
+        <v>1</v>
+      </c>
+      <c r="X32" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y32" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z32" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD32" t="b">
+        <v>1</v>
+      </c>
+      <c r="AF32" t="inlineStr">
+        <is>
+          <t>964b903e31486376a95b3a9b7b182d72568a50e195ee17dd24960fa3b4cc9c2f</t>
+        </is>
+      </c>
+      <c r="AJ32" t="inlineStr">
+        <is>
+          <t>candidates_v3_altnews.jsonl</t>
+        </is>
+      </c>
+      <c r="AK32" t="inlineStr">
+        <is>
+          <t>2026-09-07T14:32:00.027400+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>item-0032</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>validation</t>
+        </is>
+      </c>
+      <c r="D33" t="b">
+        <v>1</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>cand-ap-altnews-0567</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>https://twitter.com/JaipurDialogues/status/1980688390107590811</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>https://www.altnews.in/delhi-pollution-old-video-shared-to-claim-stubble-burning-in-punjab-is-to-be-blamed-not-diwali-crackers/</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>Liberals are blaming Diwali and fire crackers for air pollution.</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>altnews.in</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>https://www.altnews.in/delhi-pollution-old-video-shared-to-claim-stubble-burning-in-punjab-is-to-be-blamed-not-diwali-crackers/</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>provenance</t>
+        </is>
+      </c>
+      <c r="V33" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="W33" t="b">
+        <v>0</v>
+      </c>
+      <c r="X33" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y33" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z33" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD33" t="b">
+        <v>1</v>
+      </c>
+      <c r="AF33" t="inlineStr">
+        <is>
+          <t>6b3c402e397a12bad8a3cbbe7d7ab1c9d144b94f6724e18b87ca583f6782e990</t>
+        </is>
+      </c>
+      <c r="AJ33" t="inlineStr">
+        <is>
+          <t>candidates_v3_altnews.jsonl</t>
+        </is>
+      </c>
+      <c r="AK33" t="inlineStr">
+        <is>
+          <t>2026-09-07T14:36:53.597286+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>item-0033</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>validation</t>
+        </is>
+      </c>
+      <c r="D34" t="b">
+        <v>1</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>cand-ap-altnews-0568</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>https://twitter.com/MrTiwaria/status/1980725821288632349</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>https://www.altnews.in/delhi-pollution-old-video-shared-to-claim-stubble-burning-in-punjab-is-to-be-blamed-not-diwali-crackers/</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>उदारवादी लिब्रांडु लोग वायु प्रदूषण के लिए दिवाली और पटाखों को ज़िम्मेदार ठहराएँगे।</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>altnews.in</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>https://www.altnews.in/delhi-pollution-old-video-shared-to-claim-stubble-burning-in-punjab-is-to-be-blamed-not-diwali-crackers/</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>provenance</t>
+        </is>
+      </c>
+      <c r="V34" t="n">
+        <v>0.999</v>
+      </c>
+      <c r="W34" t="b">
+        <v>0</v>
+      </c>
+      <c r="X34" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y34" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z34" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD34" t="b">
+        <v>1</v>
+      </c>
+      <c r="AF34" t="inlineStr">
+        <is>
+          <t>6b3c402e397a12bad8a3cbbe7d7ab1c9d144b94f6724e18b87ca583f6782e990</t>
+        </is>
+      </c>
+      <c r="AJ34" t="inlineStr">
+        <is>
+          <t>candidates_v3_altnews.jsonl</t>
+        </is>
+      </c>
+      <c r="AK34" t="inlineStr">
+        <is>
+          <t>2026-09-07T14:36:53.599393+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>item-0034</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>v2</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>validation</t>
+        </is>
+      </c>
+      <c r="D35" t="b">
+        <v>1</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>cand-ap-leadstories-0021</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>https://twitter.com/foxwoundband/status/1266613385862447104</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>https://leadstories.com/hoax-alert/2020/06/fact-check-atlanta-did-not-deploy-a-child-militia-during-protests.html</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>video</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>Atlanta has deployed a child militia at Lenox Mall fitted with riot shields and batons.</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>leadstories.com</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>https://leadstories.com/hoax-alert/2020/06/fact-check-atlanta-did-not-deploy-a-child-militia-during-protests.html</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>provenance</t>
+        </is>
+      </c>
+      <c r="V35" t="n">
+        <v>1</v>
+      </c>
+      <c r="W35" t="b">
+        <v>1</v>
+      </c>
+      <c r="X35" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y35" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z35" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD35" t="b">
+        <v>1</v>
+      </c>
+      <c r="AF35" t="inlineStr">
+        <is>
+          <t>4b48a848c5f05592dadb58da56db7e9f10ff3752cbef3e5d9b806519bb69c622</t>
+        </is>
+      </c>
+      <c r="AJ35" t="inlineStr">
+        <is>
+          <t>candidates_v3_leadstories.jsonl</t>
+        </is>
+      </c>
+      <c r="AK35" t="inlineStr">
+        <is>
+          <t>2026-09-07T14:37:22.560671+00:00</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3684,7 +4548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P57"/>
+  <dimension ref="A1:P65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6163,6 +7027,222 @@
         </is>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>item-0027</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>dataset_ground_truth</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Israel occupied schools and hospitals, killing 160 Iranian school girls</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>provenance</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>item-0028</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>dataset_ground_truth</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>A person who is doing brutality against a Muslim balloon seller or a crowd instead of helping takes a video?</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>provenance</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>item-0029</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>dataset_ground_truth</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>This government has mastered one thing: entertainment over governance.</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>provenance</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>item-0030</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>dataset_ground_truth</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>He's so brilliant that he can work on a computer even without switching it on!</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>provenance</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>item-0031</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>dataset_ground_truth</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Rahul Gandhi called Chhath Puja 'drama'</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>provenance</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>item-0032</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>dataset_ground_truth</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Liberals are blaming Diwali and fire crackers for air pollution.</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>provenance</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>item-0033</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>dataset_ground_truth</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>उदारवादी लिब्रांडु लोग वायु प्रदूषण के लिए दिवाली और पटाखों को ज़िम्मेदार ठहराएँगे।</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>provenance</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>item-0034</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>dataset_ground_truth</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Atlanta has deployed a child militia at Lenox Mall fitted with riot shields and batons.</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>UNVERIFIED</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>provenance</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6174,7 +7254,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O38"/>
+  <dimension ref="A1:O34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -7120,6 +8200,11 @@
           <t>cand-ap-altnews-0196</t>
         </is>
       </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>item-0027</t>
+        </is>
+      </c>
       <c r="C15" t="inlineStr">
         <is>
           <t>ELIGIBLE</t>
@@ -7185,6 +8270,11 @@
           <t>cand-ap-altnews-0316</t>
         </is>
       </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>item-0028</t>
+        </is>
+      </c>
       <c r="C16" t="inlineStr">
         <is>
           <t>ELIGIBLE</t>
@@ -7250,6 +8340,11 @@
           <t>cand-ap-altnews-0382</t>
         </is>
       </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>item-0029</t>
+        </is>
+      </c>
       <c r="C17" t="inlineStr">
         <is>
           <t>ELIGIBLE</t>
@@ -7315,6 +8410,11 @@
           <t>cand-ap-altnews-0407</t>
         </is>
       </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>item-0030</t>
+        </is>
+      </c>
       <c r="C18" t="inlineStr">
         <is>
           <t>ELIGIBLE</t>
@@ -7380,6 +8480,11 @@
           <t>cand-ap-altnews-0522</t>
         </is>
       </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>item-0031</t>
+        </is>
+      </c>
       <c r="C19" t="inlineStr">
         <is>
           <t>ELIGIBLE</t>
@@ -7445,6 +8550,11 @@
           <t>cand-ap-altnews-0567</t>
         </is>
       </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>item-0032</t>
+        </is>
+      </c>
       <c r="C20" t="inlineStr">
         <is>
           <t>ELIGIBLE</t>
@@ -7510,6 +8620,11 @@
           <t>cand-ap-altnews-0568</t>
         </is>
       </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>item-0033</t>
+        </is>
+      </c>
       <c r="C21" t="inlineStr">
         <is>
           <t>ELIGIBLE</t>
@@ -7703,6 +8818,11 @@
       <c r="A24" t="inlineStr">
         <is>
           <t>cand-ap-leadstories-0021</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>item-0034</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -7834,7 +8954,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>cand-ap-leadstories-0112</t>
+          <t>cand-ap-leadstories-0212</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -7854,12 +8974,12 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=2klmuggOElE</t>
+          <t>https://www.youtube.com/watch?v=J0CLMqpsrgY</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://leadstories.com/hoax-alert/2020/06/fact-check-22-point-meme-is-mix-of-false-truth-opinion.html</t>
+          <t>https://leadstories.com/hoax-alert/2020/07/fact-check-doctors-do-recommend-vitamins-and-sunlight-for-peoples-health.html</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -7869,7 +8989,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-09-07T14:51:51.927886+00:00</t>
+          <t>2026-09-07T15:05:48.862967+00:00</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -7878,7 +8998,7 @@
         </is>
       </c>
       <c r="K26" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
@@ -7887,19 +9007,19 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>The Queen has promised the nation that better days are ahead, during a special address on Sunday.</t>
+          <t>'almost no evidence' is a misrepresentation of Dr Belchetz statement that 'there are many studies showing benefits to taking vitamins and supplements', according to the CBC article.</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t xml:space="preserve">llama3.2 (conf=1.00): </t>
+          <t>llama3.2 (conf=0.90): The original claim made in this post's caption states that 'almost no evidence backs up claims from vitamin and supplement industry'. However, according to Dr Belchetz' statement cited on YouTube (referenced by the same source as CBC article), there are many studies showing benefits of taking vitamins. The use of the term "almost" is misleading because it implies a lack of any evidence when in fact multiple researches support its claims.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>cand-ap-leadstories-0149</t>
+          <t>cand-ap-leadstories-0223</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -7914,17 +9034,17 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>facebook</t>
+          <t>youtube</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/watch/?v=251364862815976</t>
+          <t>https://www.youtube.com/watch?v=ad1ysX2iLmA</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://leadstories.com/hoax-alert/2020/06/fact-check-brooklyn-subway-attack-not-related-to-black-lives-matter-protests.html</t>
+          <t>https://leadstories.com/hoax-alert/2020/07/fact-check-birth-certificate-does-not-prove-donald-trump-had-son-with-ghislaine-maxwell.html</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -7934,7 +9054,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-09-07T14:58:31.251937+00:00</t>
+          <t>2026-09-07T15:08:10.465015+00:00</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
@@ -7952,19 +9072,19 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>#BlackLivesMatter attacking innocent white woman.</t>
+          <t>The @realJimmyTrump account has recently changed its photo from a picture of Kieran Culkin to the Birth Certificate and a meme image known as "Zuckertrump." The identity of Rogue WH Snr Advisor remains unknown, but they are most certainly not the son of President Trump and Ghislaine Maxwell.</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>llama3.2 (conf=1.00): The post's caption directly states that #BlackLivesMatter is 'attacking' an innocent white woman. The phrase suggests a causal relationship between BLM protests and the attack on Oct. 23, 2019. However, according to the article, there was no connection between Thompson's actions (a repeat transit offender) and Black Lives Matter.</t>
+          <t>llama3.2 (conf=1.00): The post's caption changes the image on @realJimmyTrump account from a picture of Kieran Culkin to one that includes the Birth Certificate with 'Zuckertrump' meme, which is an edited version of Donald Trump and implies he was involved in some scandalous activity (sex offender) but does not state it directly. The post's caption also says Rogue WH Snr Advisor are most certainly NOT Ghislaine Maxwell &amp; President trump son - making this claim MISINFORMATION_SOURCE.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>cand-ap-leadstories-0177</t>
+          <t>cand-ap-leadstories-0245</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -7984,12 +9104,12 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=1YJsxMcAJoA</t>
+          <t>https://www.youtube.com/watch?v=TYfXE8QeFHE</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://leadstories.com/hoax-alert/2020/06/fact-check-nbc-news-did-not-report-all-americans-will-receive-a-microchip-implant-by-the-end-of-the-year.html</t>
+          <t>https://leadstories.com/hoax-alert/2020/07/fact-check-clark-hunt-did-not-threaten-to-fire-his-players-and-staff-if-they-dont-stand-for-the-national-anthem.html</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -7999,7 +9119,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-09-07T15:01:38.903001+00:00</t>
+          <t>2026-09-07T15:09:56.550526+00:00</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -8008,28 +9128,28 @@
         </is>
       </c>
       <c r="K28" t="n">
-        <v>0.9999</v>
+        <v>1</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>UNVERIFIED</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>Coverage under Obamacare will require an implantable microchip?</t>
+          <t>'You are all simply paid performers on a stage and that field is my stage! You will stand, with your hand over your heart and with respect, when our Country's National Anthem is being played or you will no longer be a Kansas City Chief, a Coach for the Kansas City Chiefs or have any association with the Chiefs Organization!'</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t xml:space="preserve">llama3.2 (conf=1.00): </t>
+          <t>llama3.2 (conf=1.00): The caption of this YouTube post is identical to the claim mentioned at the beginning of the fact-check article, which was debunked as a false attribution to Clark Hunt and other NFL owners.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>cand-ap-leadstories-0184</t>
+          <t>cand-ap-leadstories-0273</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -8044,17 +9164,17 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>x</t>
+          <t>youtube</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://twitter.com/SteveGuest/status/1276221457467609091</t>
+          <t>https://www.youtube.com/watch?v=WvKSy1bwT70</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://leadstories.com/hoax-alert/2020/06/fact-check-biden-quotes-wrong-number-of-american-covid19-deaths-not-over-120-million.html</t>
+          <t>https://leadstories.com/hoax-alert/2020/07/fact-check-the-cdc-does-recommend-buying-and-using-face-masks-even-if-you-are-healthy.html</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -8064,7 +9184,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-09-07T15:04:01.666025+00:00</t>
+          <t>2026-09-07T15:17:06.077762+00:00</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -8082,19 +9202,19 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>over 120 million people died in the United States from COVID-19.</t>
+          <t>Yes, this is a real flyer,</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t xml:space="preserve">llama3.2 (conf=1.00): </t>
+          <t>llama3.2 (conf=1.00): The post's caption states that President Trump announced the CDC is changing its guidelines to recommend people wear simple cloth face masks, which includes a claim about healthy individuals not needing to buy or use face masks. This matches with what was stated in an outdated Delaware Health and Social Services infographic published March 2020.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>cand-ap-leadstories-0211</t>
+          <t>cand-ap-leadstories-0314</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -8114,12 +9234,12 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=E94pqy2rB7g</t>
+          <t>https://www.youtube.com/watch?v=VhirLohgDRc</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://leadstories.com/hoax-alert/2020/07/fact-check-doctors-do-recommend-vitamins-and-sunlight-for-peoples-health.html</t>
+          <t>https://leadstories.com/hoax-alert/2020/07/fact-check-no-evidence-european-royals-are-hunting-naked-children-for-fun-at-human-hunting-parties.html</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -8129,7 +9249,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-09-07T15:05:48.860472+00:00</t>
+          <t>2026-09-07T15:25:59.766110+00:00</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -8145,17 +9265,26 @@
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr"/>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>European royals killing naked children for fun at human hunting parties.</t>
+        </is>
+      </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>llama3.2 (conf=1.00): The claim in the Facebook post is that 'no doctor on TV tells us to strengthen our immune system: vitamins, eat right, sunlight.' However, according to the fact-check article, this claim has been debunked as false. The CDC recommends various nutrients and spending time outdoors for overall health benefits, which contradicts the idea presented by the meme.</t>
+          <t>llama3.2 (conf=1.00): The caption of this YouTube post directly links to the same source (Kevin Annetts' blog) which originally published and promoted the debunked claim. The text itself is a direct copy from Kevin Annett's video, making no distinction between fact or fiction.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>cand-ap-leadstories-0212</t>
+          <t>cand-mass-0027</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>item-0019</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -8165,127 +9294,107 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>leadstories.com</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>youtube</t>
+          <t>altnews.in</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=J0CLMqpsrgY</t>
+          <t>https://www.instagram.com/reel/DX7LBwesE-o/</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://leadstories.com/hoax-alert/2020/07/fact-check-doctors-do-recommend-vitamins-and-sunlight-for-peoples-health.html</t>
+          <t>https://www.altnews.in/bjp-media-outlets-share-holi-video-as-people-celebrating-bjp-victory-in-bengal/</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>candidates_v3_leadstories.jsonl</t>
+          <t>candidates_v2.jsonl</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-09-07T15:05:48.862967+00:00</t>
+          <t>2026-08-18T00:59:01.077843+00:00</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>DISCOVERED -&gt; SOCIAL_REFERENCE_FOUND -&gt; MEDIA_RETRIEVABLE -&gt; GROUND_TRUTH_VERIFIED -&gt; ELIGIBLE</t>
-        </is>
-      </c>
-      <c r="K31" t="n">
-        <v>0.9</v>
+          <t>DISCOVERED -&gt; ARTICLE_FOUND -&gt; SOCIAL_REFERENCE_FOUND -&gt; MEDIA_RETRIEVABLE -&gt; GROUND_TRUTH_VERIFIED -&gt; ELIGIBLE</t>
+        </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>UNVERIFIED</t>
+          <t>False claim: The post's own caption asserts that it depicts people celebrating a political event (BJP victory), but actually shows a pre-election celebration during Holi.</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>'almost no evidence' is a misrepresentation of Dr Belchetz statement that 'there are many studies showing benefits to taking vitamins and supplements', according to the CBC article.</t>
+          <t>Celebrations of Jai Sri Ram at the Holi celebrations in Kolkata, which took place two months before May 4th</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>llama3.2 (conf=0.90): The original claim made in this post's caption states that 'almost no evidence backs up claims from vitamin and supplement industry'. However, according to Dr Belchetz' statement cited on YouTube (referenced by the same source as CBC article), there are many studies showing benefits of taking vitamins. The use of the term "almost" is misleading because it implies a lack of any evidence when in fact multiple researches support its claims.</t>
+          <t>llama3.2 judge (confidence=0.90): The Instagram Post’s Own Caption Asserts the False Claim</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>cand-ap-leadstories-0223</t>
+          <t>cand-mass-0088</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ELIGIBLE</t>
+          <t>REJECTED</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>leadstories.com</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>youtube</t>
+          <t>altnews.in</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=ad1ysX2iLmA</t>
+          <t>https://www.instagram.com/reel/DPcCJWxga06/</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://leadstories.com/hoax-alert/2020/07/fact-check-birth-certificate-does-not-prove-donald-trump-had-son-with-ghislaine-maxwell.html</t>
+          <t>https://www.altnews.in/yogi-adityanath-left-to-hear-criticism-of-govt-while-ravi-kishan-was-enjoying-doctored-video-viral/</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>candidates_v3_leadstories.jsonl</t>
+          <t>candidates_v2.jsonl</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>2026-09-07T15:08:10.465015+00:00</t>
+          <t>2026-08-18T01:51:54.674020+00:00</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>DISCOVERED -&gt; SOCIAL_REFERENCE_FOUND -&gt; MEDIA_RETRIEVABLE -&gt; GROUND_TRUTH_VERIFIED -&gt; ELIGIBLE</t>
-        </is>
-      </c>
-      <c r="K32" t="n">
-        <v>1</v>
-      </c>
-      <c r="L32" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="M32" t="inlineStr">
-        <is>
-          <t>The @realJimmyTrump account has recently changed its photo from a picture of Kieran Culkin to the Birth Certificate and a meme image known as "Zuckertrump." The identity of Rogue WH Snr Advisor remains unknown, but they are most certainly not the son of President Trump and Ghislaine Maxwell.</t>
-        </is>
-      </c>
-      <c r="N32" t="inlineStr">
-        <is>
-          <t>llama3.2 (conf=1.00): The post's caption changes the image on @realJimmyTrump account from a picture of Kieran Culkin to one that includes the Birth Certificate with 'Zuckertrump' meme, which is an edited version of Donald Trump and implies he was involved in some scandalous activity (sex offender) but does not state it directly. The post's caption also says Rogue WH Snr Advisor are most certainly NOT Ghislaine Maxwell &amp; President trump son - making this claim MISINFORMATION_SOURCE.</t>
+          <t>DISCOVERED -&gt; ARTICLE_FOUND -&gt; SOCIAL_REFERENCE_FOUND -&gt; MEDIA_RETRIEVABLE -&gt; REJECTED</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr"/>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Judged NOT the misinformation source (confidence=1.00): </t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>cand-ap-leadstories-0245</t>
+          <t>cand-thequint-0182</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>item-0021</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -8295,41 +9404,33 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>leadstories.com</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>youtube</t>
+          <t>thequint.com</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=TYfXE8QeFHE</t>
+          <t>https://www.instagram.com/reel/DRmx_YwjN7Y/</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://leadstories.com/hoax-alert/2020/07/fact-check-clark-hunt-did-not-threaten-to-fire-his-players-and-staff-if-they-dont-stand-for-the-national-anthem.html</t>
+          <t>https://www.thequint.com/news/webqoof/ai-generated-yogi-lifting-weighting-without-his-hands-fact-check</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>candidates_v3_leadstories.jsonl</t>
+          <t>candidates_v2_mass_thequint.jsonl</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2026-09-07T15:09:56.550526+00:00</t>
+          <t>2026-08-18T05:29:58.023010+00:00</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>DISCOVERED -&gt; SOCIAL_REFERENCE_FOUND -&gt; MEDIA_RETRIEVABLE -&gt; GROUND_TRUTH_VERIFIED -&gt; ELIGIBLE</t>
-        </is>
-      </c>
-      <c r="K33" t="n">
-        <v>1</v>
+          <t>DISCOVERED -&gt; SOCIAL_REFERENCE_FOUND -&gt; MEDIA_RETRIEVABLE -&gt; ELIGIBLE</t>
+        </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
@@ -8338,19 +9439,24 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>'You are all simply paid performers on a stage and that field is my stage! You will stand, with your hand over your heart and with respect, when our Country's National Anthem is being played or you will no longer be a Kansas City Chief, a Coach for the Kansas City Chiefs or have any association with the Chiefs Organization!'</t>
+          <t>INDIAN YOGI MOVES 95 Kgs of weight in the gym with his mind!</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>llama3.2 (conf=1.00): The caption of this YouTube post is identical to the claim mentioned at the beginning of the fact-check article, which was debunked as a false attribution to Clark Hunt and other NFL owners.</t>
+          <t>llama3.2 judge (confidence=1.00): The caption text itself makes a specific false assertion about lifting '130 kgs' (not mentioned) and claims that it's done using one's 'mind', which is the exact same claim being debunked in the article.. NOT yet human/manual-reviewed.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>cand-ap-leadstories-0247</t>
+          <t>cand-vishvas-1173</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>item-0022</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -8360,287 +9466,45 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>leadstories.com</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>youtube</t>
+          <t>vishvasnews.com</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/watch?v=xKPWngYf2Wk</t>
+          <t>https://www.instagram.com/reel/C3tynQjr_wI/</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://leadstories.com/hoax-alert/2020/07/fact-check-doctors-claim-that-no-one-has-died-from-the-coronavirus-is-not-true.html</t>
+          <t>https://www.vishvasnews.com/politics/fact-check-akhilesh-yadav-old-video-from-kanpur-is-being-shared-as-meeting-farmers-in-delhi/</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>candidates_v3_leadstories.jsonl</t>
+          <t>candidates_v2_mass_vishvas.jsonl</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>2026-09-07T15:10:29.017026+00:00</t>
+          <t>2026-08-18T10:12:40.325601+00:00</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>DISCOVERED -&gt; SOCIAL_REFERENCE_FOUND -&gt; MEDIA_RETRIEVABLE -&gt; GROUND_TRUTH_VERIFIED -&gt; ELIGIBLE</t>
-        </is>
-      </c>
-      <c r="K34" t="n">
-        <v>1</v>
+          <t>DISCOVERED -&gt; SOCIAL_REFERENCE_FOUND -&gt; MEDIA_RETRIEVABLE -&gt; ELIGIBLE -&gt; UNRESOLVED -&gt; ELIGIBLE</t>
+        </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>UNVERIFIED</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>The World Health Organization (WHO) has officially declared the outbreak of novel coronavirus disease, COVID-19, a pandemic.</t>
+          <t>अखिलेश यादव किसानों से मिलने दिल्ली पहुंचे।</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">llama3.2 (conf=1.00): </t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>cand-mass-0027</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>item-0019</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>ELIGIBLE</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>altnews.in</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/reel/DX7LBwesE-o/</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>https://www.altnews.in/bjp-media-outlets-share-holi-video-as-people-celebrating-bjp-victory-in-bengal/</t>
-        </is>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>candidates_v2.jsonl</t>
-        </is>
-      </c>
-      <c r="I35" t="inlineStr">
-        <is>
-          <t>2026-08-18T00:59:01.077843+00:00</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>DISCOVERED -&gt; ARTICLE_FOUND -&gt; SOCIAL_REFERENCE_FOUND -&gt; MEDIA_RETRIEVABLE -&gt; GROUND_TRUTH_VERIFIED -&gt; ELIGIBLE</t>
-        </is>
-      </c>
-      <c r="L35" t="inlineStr">
-        <is>
-          <t>False claim: The post's own caption asserts that it depicts people celebrating a political event (BJP victory), but actually shows a pre-election celebration during Holi.</t>
-        </is>
-      </c>
-      <c r="M35" t="inlineStr">
-        <is>
-          <t>Celebrations of Jai Sri Ram at the Holi celebrations in Kolkata, which took place two months before May 4th</t>
-        </is>
-      </c>
-      <c r="N35" t="inlineStr">
-        <is>
-          <t>llama3.2 judge (confidence=0.90): The Instagram Post’s Own Caption Asserts the False Claim</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>cand-mass-0088</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>REJECTED</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>altnews.in</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/reel/DPcCJWxga06/</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>https://www.altnews.in/yogi-adityanath-left-to-hear-criticism-of-govt-while-ravi-kishan-was-enjoying-doctored-video-viral/</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>candidates_v2.jsonl</t>
-        </is>
-      </c>
-      <c r="I36" t="inlineStr">
-        <is>
-          <t>2026-08-18T01:51:54.674020+00:00</t>
-        </is>
-      </c>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>DISCOVERED -&gt; ARTICLE_FOUND -&gt; SOCIAL_REFERENCE_FOUND -&gt; MEDIA_RETRIEVABLE -&gt; REJECTED</t>
-        </is>
-      </c>
-      <c r="N36" t="inlineStr"/>
-      <c r="O36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Judged NOT the misinformation source (confidence=1.00): </t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>cand-thequint-0182</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>item-0021</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>ELIGIBLE</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>thequint.com</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/reel/DRmx_YwjN7Y/</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>https://www.thequint.com/news/webqoof/ai-generated-yogi-lifting-weighting-without-his-hands-fact-check</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>candidates_v2_mass_thequint.jsonl</t>
-        </is>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>2026-08-18T05:29:58.023010+00:00</t>
-        </is>
-      </c>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>DISCOVERED -&gt; SOCIAL_REFERENCE_FOUND -&gt; MEDIA_RETRIEVABLE -&gt; ELIGIBLE</t>
-        </is>
-      </c>
-      <c r="L37" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="M37" t="inlineStr">
-        <is>
-          <t>INDIAN YOGI MOVES 95 Kgs of weight in the gym with his mind!</t>
-        </is>
-      </c>
-      <c r="N37" t="inlineStr">
-        <is>
-          <t>llama3.2 judge (confidence=1.00): The caption text itself makes a specific false assertion about lifting '130 kgs' (not mentioned) and claims that it's done using one's 'mind', which is the exact same claim being debunked in the article.. NOT yet human/manual-reviewed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>cand-vishvas-1173</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>item-0022</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>ELIGIBLE</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>vishvasnews.com</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>https://www.instagram.com/reel/C3tynQjr_wI/</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>https://www.vishvasnews.com/politics/fact-check-akhilesh-yadav-old-video-from-kanpur-is-being-shared-as-meeting-farmers-in-delhi/</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>candidates_v2_mass_vishvas.jsonl</t>
-        </is>
-      </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>2026-08-18T10:12:40.325601+00:00</t>
-        </is>
-      </c>
-      <c r="J38" t="inlineStr">
-        <is>
-          <t>DISCOVERED -&gt; SOCIAL_REFERENCE_FOUND -&gt; MEDIA_RETRIEVABLE -&gt; ELIGIBLE -&gt; UNRESOLVED -&gt; ELIGIBLE</t>
-        </is>
-      </c>
-      <c r="L38" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="M38" t="inlineStr">
-        <is>
-          <t>अखिलेश यादव किसानों से मिलने दिल्ली पहुंचे।</t>
-        </is>
-      </c>
-      <c r="N38" t="inlineStr">
         <is>
           <t>llama3.2 judge (confidence=1.00): The caption text itself makes the specific false assertion that 'अखिलेश यादव' is meeting with farmers in Delhi, which contradicts the fact-check article's conclusion.. NOT yet human/manual-reviewed.</t>
         </is>
@@ -8657,7 +9521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B68"/>
+  <dimension ref="A1:B71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -8684,7 +9548,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-07T15:17:01+00:00</t>
+          <t>2026-09-07T15:38:20+00:00</t>
         </is>
       </c>
     </row>
@@ -8695,7 +9559,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4">
@@ -8715,7 +9579,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>17</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6">
@@ -8757,55 +9621,55 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">    MISLEADING</t>
+          <t xml:space="preserve">    UNVERIFIED</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">    TRUE</t>
+          <t xml:space="preserve">    MISLEADING</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>--- platform distribution ---</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr"/>
+          <t xml:space="preserve">    TRUE</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">    instagram</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>13</v>
-      </c>
+          <t>--- platform distribution ---</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">    (none)</t>
+          <t xml:space="preserve">    instagram</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="16">
@@ -8815,155 +9679,155 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>--- language distribution ---</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr"/>
+          <t xml:space="preserve">    (none)</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">    en</t>
+          <t xml:space="preserve">    facebook</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">    hi</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>3</v>
-      </c>
+          <t>--- language distribution ---</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">    hi-en-mixed</t>
+          <t xml:space="preserve">    en</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1</v>
+        <v>30</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>--- split distribution ---</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr"/>
+          <t xml:space="preserve">    hi</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">    validation</t>
+          <t xml:space="preserve">    hi-en-mixed</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">    (none)</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>9</v>
-      </c>
+          <t>--- split distribution ---</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>--- benchmark_version distribution ---</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr"/>
+          <t xml:space="preserve">    validation</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">    v2</t>
+          <t xml:space="preserve">    (none)</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">    v1</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>9</v>
-      </c>
+          <t>--- benchmark_version distribution ---</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>--- claim_type distribution ---</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr"/>
+          <t xml:space="preserve">    v2</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">    provenance</t>
+          <t xml:space="preserve">    v1</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>21</v>
+        <v>9</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">    misleading_context</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>2</v>
-      </c>
+          <t>--- claim_type distribution ---</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">    visual</t>
+          <t xml:space="preserve">    provenance</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1</v>
+        <v>29</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">    event</t>
+          <t xml:space="preserve">    misleading_context</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">    quote</t>
+          <t xml:space="preserve">    visual</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -8973,103 +9837,103 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>--- media (video/photo) distribution ---</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr"/>
+          <t xml:space="preserve">    event</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">    video</t>
+          <t xml:space="preserve">    quote</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">    photo</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>3</v>
-      </c>
+          <t>--- media (video/photo) distribution ---</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>--- factchecker distribution ---</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr"/>
+          <t xml:space="preserve">    video</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>31</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">    altnews.in</t>
+          <t xml:space="preserve">    photo</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">    boomlive.in</t>
-        </is>
-      </c>
-      <c r="B38" t="n">
-        <v>4</v>
-      </c>
+          <t>--- factchecker distribution ---</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">    tier-1-source:boomlive.in</t>
+          <t xml:space="preserve">    altnews.in</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">    tier-1-source:altnews.in</t>
+          <t xml:space="preserve">    boomlive.in</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">    tier-1-source:factly.in</t>
+          <t xml:space="preserve">    tier-1-source:boomlive.in</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">    tier-1-source:boomlive.in (hindi.boomlive.in)</t>
+          <t xml:space="preserve">    tier-1-source:altnews.in</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">    tier-1-source:altnews.in (hindi.altnews.in)</t>
+          <t xml:space="preserve">    tier-1-source:factly.in</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -9079,7 +9943,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">    thequint.com</t>
+          <t xml:space="preserve">    tier-1-source:boomlive.in (hindi.boomlive.in)</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -9089,7 +9953,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">    vishvasnews.com</t>
+          <t xml:space="preserve">    tier-1-source:altnews.in (hindi.altnews.in)</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -9099,35 +9963,37 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>--- ground-truth tier distribution ---</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr"/>
+          <t xml:space="preserve">    thequint.com</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">    (none)</t>
+          <t xml:space="preserve">    vishvasnews.com</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">    1</t>
+          <t xml:space="preserve">    leadstories.com</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>--- difficulty distribution ---</t>
+          <t>--- ground-truth tier distribution ---</t>
         </is>
       </c>
       <c r="B49" t="inlineStr"/>
@@ -9139,41 +10005,41 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>--- annotation_status distribution ---</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr"/>
+          <t xml:space="preserve">    1</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve">    (none)</t>
-        </is>
-      </c>
-      <c r="B52" t="n">
-        <v>17</v>
-      </c>
+          <t>--- difficulty distribution ---</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">    tier1_professional</t>
+          <t xml:space="preserve">    (none)</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>9</v>
+        <v>34</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>--- modality availability (true count) ---</t>
+          <t>--- annotation_status distribution ---</t>
         </is>
       </c>
       <c r="B54" t="inlineStr"/>
@@ -9181,75 +10047,75 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">    audio_available</t>
+          <t xml:space="preserve">    (none)</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>13</v>
+        <v>25</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">    ocr_available</t>
+          <t xml:space="preserve">    tier1_professional</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">    caption_available</t>
-        </is>
-      </c>
-      <c r="B57" t="n">
-        <v>16</v>
-      </c>
+          <t>--- modality availability (true count) ---</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">    visual_information_available</t>
+          <t xml:space="preserve">    audio_available</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>--- cross-post ---</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr"/>
+          <t xml:space="preserve">    ocr_available</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t xml:space="preserve">    cross_post_possible = true</t>
+          <t xml:space="preserve">    caption_available</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>17</v>
+        <v>24</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t xml:space="preserve">    cross_post_verified = true</t>
+          <t xml:space="preserve">    visual_information_available</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>--- missing-field rates ---</t>
+          <t>--- cross-post ---</t>
         </is>
       </c>
       <c r="B62" t="inlineStr"/>
@@ -9257,72 +10123,100 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t xml:space="preserve">    no factcheck_url</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>0/26 (0%)</t>
-        </is>
+          <t xml:space="preserve">    cross_post_possible = true</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t xml:space="preserve">    no publication_date</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>17/26 (65%)</t>
-        </is>
+          <t xml:space="preserve">    cross_post_verified = true</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t xml:space="preserve">    no media_hash</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>9/26 (34%)</t>
-        </is>
-      </c>
+          <t>--- missing-field rates ---</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t xml:space="preserve">    no split</t>
+          <t xml:space="preserve">    no factcheck_url</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>9/26 (34%)</t>
+          <t>0/34 (0%)</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t xml:space="preserve">    no difficulty</t>
+          <t xml:space="preserve">    no publication_date</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>26/26 (100%)</t>
+          <t>25/34 (73%)</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
+          <t xml:space="preserve">    no media_hash</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>9/34 (26%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    no split</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>9/34 (26%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    no difficulty</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>34/34 (100%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
           <t xml:space="preserve">    no candidate_id (provenance)</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>9/26 (34%)</t>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>9/34 (26%)</t>
         </is>
       </c>
     </row>
@@ -11379,9 +12273,13 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>item-0032, item-0033</t>
+        </is>
+      </c>
       <c r="E12" t="inlineStr">
         <is>
           <t>same content_hash on &gt;1 item -- repost/cross-post; keep + flag, do not delete</t>

</xml_diff>